<commit_message>
add patient tracker exporter to generate landscape PDF tables and TSV reports for clinical metrics
</commit_message>
<xml_diff>
--- a/core/UAT Plan.xlsx
+++ b/core/UAT Plan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Demo person 1" sheetId="1" state="visible" r:id="rId4"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
   <si>
     <t xml:space="preserve">Test Case #</t>
   </si>
@@ -554,13 +554,64 @@
   </si>
   <si>
     <t xml:space="preserve">Requires documented alarm symptoms (dysphagia, odynophagia, unexplained weight loss, hematemesis, melena) OR failed conservative treatment (PPI trial min. 4–8 weeks). Rejection issued when only vague, non-specific symptoms are present with no prior workup.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 14</t>
+  </si>
+  <si>
+    <t>J0885</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Injection, epoetin alfa (for non-ESRD use), 1000 units</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient: Robert Hayes, 67M, Oncology Follow-up Visit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient with chemotherapy-induced anemia secondary to metastatic lung cancer. Hemoglobin level documented at 8.7 g/dL. Active chemotherapy regimen noted in encounter documentation. Prior epoetin response documented. Supporting CBC labs attached.</t>
+  </si>
+  <si>
+    <t>Approval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior authorization required. Documentation must include active chemotherapy treatment, recent hemoglobin lab values, anemia diagnosis, and provider treatment plan supporting epoetin alfa use.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient: Melissa Turner, 52F, Outpatient Hematology Visit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Request submitted for fatigue complaints without confirmed anemia diagnosis. Hemoglobin value missing from records. No evidence of chemotherapy, CKD-related indication, or transfusion history. Incomplete clinical notes uploaded.</t>
+  </si>
+  <si>
+    <t>Rejection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior authorization denied due to insufficient clinical documentation. Missing qualifying diagnosis, lab results, and medical necessity criteria for epoetin alfa therapy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient: Daniel Brooks, 61M, Chronic Disease Management Encounter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient with myelodysplastic syndrome and symptomatic anemia. Hemoglobin documented at 9.9 g/dL. History of partial response to ESA therapy. Provider submitted supporting labs, but transferrin saturation and ferritin studies are pending review.</t>
+  </si>
+  <si>
+    <t>Moderate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior authorization placed in pending/moderate review status. Additional documentation requested including iron studies, treatment history, and confirmation of ongoing anemia management protocol.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -587,6 +638,12 @@
       <sz val="12.000000"/>
       <name val="Times"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12.000000"/>
+      <color indexed="64"/>
+      <name val="Times"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -606,7 +663,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -656,19 +713,45 @@
       <diagonal style="none"/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="none"/>
+      <right style="none"/>
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom/>
-      <diagonal/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="59">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -734,18 +817,12 @@
     <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf fontId="0" fillId="3" borderId="2" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="3" borderId="2" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -815,11 +892,38 @@
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf fontId="2" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1735,7 +1839,7 @@
       <c r="A3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="23"/>
+      <c r="B3" s="2"/>
       <c r="C3" s="9"/>
       <c r="D3" s="11"/>
       <c r="E3" s="11" t="s">
@@ -1757,7 +1861,7 @@
       <c r="A4" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="23"/>
+      <c r="B4" s="2"/>
       <c r="C4" s="9">
         <v>36558</v>
       </c>
@@ -1785,7 +1889,7 @@
       <c r="A5" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="23"/>
+      <c r="B5" s="2"/>
       <c r="C5" s="9"/>
       <c r="D5" s="11"/>
       <c r="E5" s="11" t="s">
@@ -1807,7 +1911,7 @@
       <c r="A6" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="23"/>
+      <c r="B6" s="2"/>
       <c r="C6" s="8">
         <v>50360</v>
       </c>
@@ -1835,7 +1939,7 @@
       <c r="A7" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="23"/>
+      <c r="B7" s="2"/>
       <c r="C7" s="8"/>
       <c r="D7" s="17"/>
       <c r="E7" s="17" t="s">
@@ -1857,7 +1961,7 @@
       <c r="A8" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="23"/>
+      <c r="B8" s="2"/>
       <c r="C8" s="8">
         <v>50394</v>
       </c>
@@ -1885,7 +1989,7 @@
       <c r="A9" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="23"/>
+      <c r="B9" s="2"/>
       <c r="C9" s="8"/>
       <c r="D9" s="17"/>
       <c r="E9" s="17" t="s">
@@ -1907,7 +2011,7 @@
       <c r="A10" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="23"/>
+      <c r="B10" s="2"/>
       <c r="C10" s="8">
         <v>77012</v>
       </c>
@@ -1935,7 +2039,7 @@
       <c r="A11" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="23"/>
+      <c r="B11" s="2"/>
       <c r="C11" s="8"/>
       <c r="D11" s="17"/>
       <c r="E11" s="17" t="s">
@@ -1957,11 +2061,11 @@
       <c r="A12" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="23"/>
-      <c r="C12" s="24">
+      <c r="B12" s="2"/>
+      <c r="C12" s="23">
         <v>36558</v>
       </c>
-      <c r="D12" s="25" t="s">
+      <c r="D12" s="24" t="s">
         <v>51</v>
       </c>
       <c r="E12" s="11" t="s">
@@ -1973,7 +2077,7 @@
       <c r="G12" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="H12" s="25" t="s">
+      <c r="H12" s="24" t="s">
         <v>53</v>
       </c>
       <c r="I12" s="1">
@@ -1984,7 +2088,7 @@
       <c r="A13" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="B13" s="23"/>
+      <c r="B13" s="2"/>
       <c r="C13" s="9"/>
       <c r="D13" s="11"/>
       <c r="E13" s="11" t="s">
@@ -2002,14 +2106,14 @@
       </c>
     </row>
     <row r="14" ht="28.5">
-      <c r="A14" s="26" t="s">
+      <c r="A14" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B14" s="23"/>
-      <c r="C14" s="24">
+      <c r="B14" s="2"/>
+      <c r="C14" s="23">
         <v>90999</v>
       </c>
-      <c r="D14" s="25" t="s">
+      <c r="D14" s="24" t="s">
         <v>45</v>
       </c>
       <c r="E14" s="11" t="s">
@@ -2021,7 +2125,7 @@
       <c r="G14" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="H14" s="25" t="s">
+      <c r="H14" s="24" t="s">
         <v>48</v>
       </c>
       <c r="I14" s="1">
@@ -2029,10 +2133,10 @@
       </c>
     </row>
     <row r="15" ht="28.5">
-      <c r="A15" s="26" t="s">
+      <c r="A15" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B15" s="23"/>
+      <c r="B15" s="2"/>
       <c r="C15" s="9"/>
       <c r="D15" s="11"/>
       <c r="E15" s="11" t="s">
@@ -2050,14 +2154,14 @@
       </c>
     </row>
     <row r="16" ht="14.25">
-      <c r="A16" s="26" t="s">
+      <c r="A16" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B16" s="23"/>
-      <c r="C16" s="24">
+      <c r="B16" s="2"/>
+      <c r="C16" s="23">
         <v>36558</v>
       </c>
-      <c r="D16" s="25" t="s">
+      <c r="D16" s="24" t="s">
         <v>51</v>
       </c>
       <c r="E16" s="11" t="s">
@@ -2069,7 +2173,7 @@
       <c r="G16" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="H16" s="25" t="s">
+      <c r="H16" s="24" t="s">
         <v>53</v>
       </c>
       <c r="I16" s="1">
@@ -2080,7 +2184,7 @@
       <c r="A17" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="23"/>
+      <c r="B17" s="2"/>
       <c r="C17" s="9"/>
       <c r="D17" s="11"/>
       <c r="E17" s="11" t="s">
@@ -2098,26 +2202,26 @@
       </c>
     </row>
     <row r="18" ht="28.5">
-      <c r="A18" s="26" t="s">
+      <c r="A18" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B18" s="23"/>
-      <c r="C18" s="27">
+      <c r="B18" s="2"/>
+      <c r="C18" s="25">
         <v>50360</v>
       </c>
-      <c r="D18" s="28" t="s">
+      <c r="D18" s="26" t="s">
         <v>56</v>
       </c>
       <c r="E18" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="F18" s="29" t="s">
+      <c r="F18" s="27" t="s">
         <v>58</v>
       </c>
       <c r="G18" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="H18" s="28" t="s">
+      <c r="H18" s="26" t="s">
         <v>59</v>
       </c>
       <c r="I18" s="1">
@@ -2125,16 +2229,16 @@
       </c>
     </row>
     <row r="19" ht="28.5">
-      <c r="A19" s="26" t="s">
+      <c r="A19" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B19" s="23"/>
+      <c r="B19" s="2"/>
       <c r="C19" s="8"/>
       <c r="D19" s="17"/>
       <c r="E19" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="F19" s="29" t="s">
+      <c r="F19" s="27" t="s">
         <v>61</v>
       </c>
       <c r="G19" s="19" t="s">
@@ -2146,14 +2250,14 @@
       </c>
     </row>
     <row r="20" ht="14.25">
-      <c r="A20" s="26" t="s">
+      <c r="A20" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B20" s="23"/>
-      <c r="C20" s="27">
+      <c r="B20" s="2"/>
+      <c r="C20" s="25">
         <v>50394</v>
       </c>
-      <c r="D20" s="28" t="s">
+      <c r="D20" s="26" t="s">
         <v>62</v>
       </c>
       <c r="E20" s="17" t="s">
@@ -2165,7 +2269,7 @@
       <c r="G20" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="H20" s="28" t="s">
+      <c r="H20" s="26" t="s">
         <v>65</v>
       </c>
       <c r="I20" s="1">
@@ -2176,7 +2280,7 @@
       <c r="A21" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B21" s="23"/>
+      <c r="B21" s="2"/>
       <c r="C21" s="8"/>
       <c r="D21" s="17"/>
       <c r="E21" s="17" t="s">
@@ -2194,14 +2298,14 @@
       </c>
     </row>
     <row r="22" ht="14.25">
-      <c r="A22" s="26" t="s">
+      <c r="A22" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B22" s="23"/>
-      <c r="C22" s="27">
+      <c r="B22" s="2"/>
+      <c r="C22" s="25">
         <v>77012</v>
       </c>
-      <c r="D22" s="28" t="s">
+      <c r="D22" s="26" t="s">
         <v>68</v>
       </c>
       <c r="E22" s="17" t="s">
@@ -2213,7 +2317,7 @@
       <c r="G22" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="H22" s="28" t="s">
+      <c r="H22" s="26" t="s">
         <v>69</v>
       </c>
       <c r="I22" s="1">
@@ -2224,7 +2328,7 @@
       <c r="A23" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B23" s="23"/>
+      <c r="B23" s="2"/>
       <c r="C23" s="8"/>
       <c r="D23" s="17"/>
       <c r="E23" s="17" t="s">
@@ -2242,7 +2346,7 @@
       </c>
     </row>
     <row r="24" ht="14.25">
-      <c r="H24" s="25"/>
+      <c r="H24" s="24"/>
     </row>
     <row r="25" ht="14.25">
       <c r="H25" s="11"/>
@@ -2337,7 +2441,7 @@
       <c r="A2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="28" t="s">
         <v>77</v>
       </c>
       <c r="C2" s="8">
@@ -2367,7 +2471,7 @@
       <c r="A3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="30"/>
+      <c r="B3" s="28"/>
       <c r="C3" s="8"/>
       <c r="D3" s="17"/>
       <c r="E3" s="17" t="s">
@@ -2389,7 +2493,7 @@
       <c r="A4" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="30"/>
+      <c r="B4" s="28"/>
       <c r="C4" s="8">
         <v>21196</v>
       </c>
@@ -2417,7 +2521,7 @@
       <c r="A5" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="30"/>
+      <c r="B5" s="28"/>
       <c r="C5" s="8"/>
       <c r="D5" s="17"/>
       <c r="E5" s="17" t="s">
@@ -2439,7 +2543,7 @@
       <c r="A6" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="30"/>
+      <c r="B6" s="28"/>
       <c r="C6" s="8">
         <v>21210</v>
       </c>
@@ -2467,7 +2571,7 @@
       <c r="A7" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="30"/>
+      <c r="B7" s="28"/>
       <c r="C7" s="8"/>
       <c r="D7" s="17"/>
       <c r="E7" s="17" t="s">
@@ -2489,7 +2593,7 @@
       <c r="A8" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="30"/>
+      <c r="B8" s="28"/>
       <c r="C8" s="8">
         <v>21085</v>
       </c>
@@ -2517,7 +2621,7 @@
       <c r="A9" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="30"/>
+      <c r="B9" s="28"/>
       <c r="C9" s="8"/>
       <c r="D9" s="17"/>
       <c r="E9" s="17" t="s">
@@ -2539,7 +2643,7 @@
       <c r="A10" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="30"/>
+      <c r="B10" s="28"/>
       <c r="C10" s="8">
         <v>21235</v>
       </c>
@@ -2567,7 +2671,7 @@
       <c r="A11" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="30"/>
+      <c r="B11" s="28"/>
       <c r="C11" s="8"/>
       <c r="D11" s="17"/>
       <c r="E11" s="17" t="s">
@@ -2618,442 +2722,442 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" style="31" width="12"/>
-    <col bestFit="1" customWidth="1" min="2" max="2" style="31" width="11.85546875"/>
-    <col min="3" max="3" style="31" width="9.140625"/>
-    <col customWidth="1" min="4" max="5" style="32" width="42.85546875"/>
-    <col customWidth="1" min="6" max="6" style="32" width="30.85546875"/>
-    <col bestFit="1" customWidth="1" min="7" max="7" style="31" width="17.5703125"/>
-    <col customWidth="1" min="8" max="8" style="32" width="46.42578125"/>
-    <col min="9" max="16384" style="31" width="9.140625"/>
+    <col customWidth="1" min="1" max="1" style="29" width="12"/>
+    <col bestFit="1" customWidth="1" min="2" max="2" style="29" width="11.85546875"/>
+    <col min="3" max="3" style="29" width="9.140625"/>
+    <col customWidth="1" min="4" max="5" style="30" width="42.85546875"/>
+    <col customWidth="1" min="6" max="6" style="30" width="30.85546875"/>
+    <col bestFit="1" customWidth="1" min="7" max="7" style="29" width="17.5703125"/>
+    <col customWidth="1" min="8" max="8" style="30" width="46.42578125"/>
+    <col min="9" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
-    <row r="1" s="33" customFormat="1">
-      <c r="A1" s="34" t="s">
+    <row r="1" s="31" customFormat="1">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="B1" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="C1" s="32" t="s">
         <v>108</v>
       </c>
-      <c r="D1" s="35" t="s">
+      <c r="D1" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="35" t="s">
+      <c r="E1" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="35" t="s">
+      <c r="F1" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="34" t="s">
+      <c r="G1" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="34" t="s">
+      <c r="H1" s="32" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" ht="57">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="35" t="s">
         <v>109</v>
       </c>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="36" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="E2" s="40" t="s">
+      <c r="E2" s="38" t="s">
         <v>112</v>
       </c>
-      <c r="F2" s="40" t="s">
+      <c r="F2" s="38" t="s">
         <v>113</v>
       </c>
-      <c r="G2" s="41" t="s">
+      <c r="G2" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="40" t="s">
+      <c r="H2" s="38" t="s">
         <v>114</v>
       </c>
-      <c r="I2" s="42">
+      <c r="I2" s="40">
         <v>260</v>
       </c>
-      <c r="J2" s="31"/>
+      <c r="J2" s="29"/>
     </row>
     <row r="3" ht="50.25" customHeight="1">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="B3" s="43"/>
-      <c r="C3" s="44"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="40" t="s">
+      <c r="B3" s="41"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="38" t="s">
         <v>115</v>
       </c>
-      <c r="F3" s="40" t="s">
+      <c r="F3" s="38" t="s">
         <v>116</v>
       </c>
-      <c r="G3" s="41" t="s">
+      <c r="G3" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="40" t="s">
+      <c r="H3" s="38" t="s">
         <v>117</v>
       </c>
-      <c r="I3" s="42">
+      <c r="I3" s="40">
         <v>261</v>
       </c>
-      <c r="J3" s="31"/>
+      <c r="J3" s="29"/>
     </row>
     <row r="4" ht="71.25">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="35" t="s">
         <v>109</v>
       </c>
-      <c r="C4" s="38" t="s">
+      <c r="C4" s="36" t="s">
         <v>118</v>
       </c>
-      <c r="D4" s="39" t="s">
+      <c r="D4" s="37" t="s">
         <v>119</v>
       </c>
-      <c r="E4" s="40" t="s">
+      <c r="E4" s="38" t="s">
         <v>120</v>
       </c>
-      <c r="F4" s="40" t="s">
+      <c r="F4" s="38" t="s">
         <v>121</v>
       </c>
-      <c r="G4" s="41" t="s">
+      <c r="G4" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="40" t="s">
+      <c r="H4" s="38" t="s">
         <v>122</v>
       </c>
-      <c r="I4" s="42">
+      <c r="I4" s="40">
         <v>262</v>
       </c>
-      <c r="J4" s="31"/>
+      <c r="J4" s="29"/>
     </row>
     <row r="5" ht="57">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="B5" s="43"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="40" t="s">
+      <c r="B5" s="41"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="38" t="s">
         <v>123</v>
       </c>
-      <c r="F5" s="40" t="s">
+      <c r="F5" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="G5" s="41" t="s">
+      <c r="G5" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="40" t="s">
+      <c r="H5" s="38" t="s">
         <v>125</v>
       </c>
-      <c r="I5" s="42">
+      <c r="I5" s="40">
         <v>263</v>
       </c>
-      <c r="J5" s="31"/>
+      <c r="J5" s="29"/>
     </row>
     <row r="6" ht="57">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="35" t="s">
         <v>109</v>
       </c>
-      <c r="C6" s="38" t="s">
+      <c r="C6" s="36" t="s">
         <v>110</v>
       </c>
-      <c r="D6" s="39" t="s">
+      <c r="D6" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="E6" s="40" t="s">
+      <c r="E6" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="F6" s="40" t="s">
+      <c r="F6" s="38" t="s">
         <v>127</v>
       </c>
-      <c r="G6" s="41" t="s">
+      <c r="G6" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="40" t="s">
+      <c r="H6" s="38" t="s">
         <v>114</v>
       </c>
-      <c r="I6" s="42">
+      <c r="I6" s="40">
         <v>264</v>
       </c>
-      <c r="J6" s="31"/>
+      <c r="J6" s="29"/>
     </row>
     <row r="7" ht="108.75">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="43"/>
-      <c r="C7" s="44"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="46" t="s">
+      <c r="B7" s="41"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="44" t="s">
         <v>128</v>
       </c>
-      <c r="F7" s="46" t="s">
+      <c r="F7" s="44" t="s">
         <v>129</v>
       </c>
-      <c r="G7" s="46" t="s">
+      <c r="G7" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="46" t="s">
+      <c r="H7" s="44" t="s">
         <v>117</v>
       </c>
-      <c r="I7" s="42">
+      <c r="I7" s="40">
         <v>265</v>
       </c>
-      <c r="J7" s="31"/>
+      <c r="J7" s="29"/>
     </row>
     <row r="8" ht="108.75">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="34" t="s">
         <v>74</v>
       </c>
-      <c r="B8" s="37" t="s">
+      <c r="B8" s="35" t="s">
         <v>109</v>
       </c>
-      <c r="C8" s="38" t="s">
+      <c r="C8" s="36" t="s">
         <v>118</v>
       </c>
-      <c r="D8" s="47" t="s">
+      <c r="D8" s="45" t="s">
         <v>119</v>
       </c>
-      <c r="E8" s="46" t="s">
+      <c r="E8" s="44" t="s">
         <v>130</v>
       </c>
-      <c r="F8" s="46" t="s">
+      <c r="F8" s="44" t="s">
         <v>131</v>
       </c>
-      <c r="G8" s="46" t="s">
+      <c r="G8" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="46" t="s">
+      <c r="H8" s="44" t="s">
         <v>122</v>
       </c>
-      <c r="I8" s="42">
+      <c r="I8" s="40">
         <v>266</v>
       </c>
-      <c r="J8" s="31"/>
+      <c r="J8" s="29"/>
     </row>
     <row r="9" ht="108.75">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="34" t="s">
         <v>74</v>
       </c>
-      <c r="B9" s="43"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="48"/>
-      <c r="E9" s="46" t="s">
+      <c r="B9" s="41"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="44" t="s">
         <v>132</v>
       </c>
-      <c r="F9" s="46" t="s">
+      <c r="F9" s="44" t="s">
         <v>133</v>
       </c>
-      <c r="G9" s="46" t="s">
+      <c r="G9" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="46" t="s">
+      <c r="H9" s="44" t="s">
         <v>125</v>
       </c>
-      <c r="I9" s="42">
+      <c r="I9" s="40">
         <v>267</v>
       </c>
-      <c r="J9" s="31"/>
+      <c r="J9" s="29"/>
     </row>
     <row r="10" ht="108.75">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="34" t="s">
         <v>75</v>
       </c>
-      <c r="B10" s="37" t="s">
+      <c r="B10" s="35" t="s">
         <v>134</v>
       </c>
-      <c r="C10" s="38" t="s">
+      <c r="C10" s="36" t="s">
         <v>135</v>
       </c>
-      <c r="D10" s="47" t="s">
+      <c r="D10" s="45" t="s">
         <v>136</v>
       </c>
-      <c r="E10" s="46" t="s">
+      <c r="E10" s="44" t="s">
         <v>137</v>
       </c>
-      <c r="F10" s="46" t="s">
+      <c r="F10" s="44" t="s">
         <v>138</v>
       </c>
-      <c r="G10" s="46" t="s">
+      <c r="G10" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="46" t="s">
+      <c r="H10" s="44" t="s">
         <v>139</v>
       </c>
-      <c r="I10" s="42">
+      <c r="I10" s="40">
         <v>268</v>
       </c>
-      <c r="J10" s="31"/>
+      <c r="J10" s="29"/>
     </row>
     <row r="11" ht="87">
-      <c r="A11" s="36" t="s">
+      <c r="A11" s="34" t="s">
         <v>75</v>
       </c>
-      <c r="B11" s="43"/>
-      <c r="C11" s="44"/>
-      <c r="D11" s="48"/>
-      <c r="E11" s="46" t="s">
+      <c r="B11" s="41"/>
+      <c r="C11" s="42"/>
+      <c r="D11" s="46"/>
+      <c r="E11" s="44" t="s">
         <v>140</v>
       </c>
-      <c r="F11" s="46" t="s">
+      <c r="F11" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="G11" s="46" t="s">
+      <c r="G11" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="46" t="s">
+      <c r="H11" s="44" t="s">
         <v>142</v>
       </c>
-      <c r="I11" s="42">
+      <c r="I11" s="40">
         <v>269</v>
       </c>
-      <c r="J11" s="31"/>
+      <c r="J11" s="29"/>
     </row>
     <row r="12" ht="71.25">
-      <c r="A12" s="42" t="s">
+      <c r="A12" s="40" t="s">
         <v>76</v>
       </c>
-      <c r="B12" s="49" t="s">
+      <c r="B12" s="47" t="s">
         <v>143</v>
       </c>
-      <c r="C12" s="42" t="s">
+      <c r="C12" s="40" t="s">
         <v>144</v>
       </c>
-      <c r="D12" s="32" t="s">
+      <c r="D12" s="30" t="s">
         <v>145</v>
       </c>
-      <c r="E12" s="32" t="s">
+      <c r="E12" s="30" t="s">
         <v>146</v>
       </c>
-      <c r="F12" s="32" t="s">
+      <c r="F12" s="30" t="s">
         <v>147</v>
       </c>
-      <c r="G12" s="41" t="s">
+      <c r="G12" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="H12" s="32" t="s">
+      <c r="H12" s="30" t="s">
         <v>142</v>
       </c>
-      <c r="I12" s="42">
+      <c r="I12" s="40">
         <v>270</v>
       </c>
     </row>
     <row r="13" ht="71.25">
-      <c r="A13" s="42" t="s">
+      <c r="A13" s="40" t="s">
         <v>76</v>
       </c>
-      <c r="B13" s="49"/>
-      <c r="C13" s="42"/>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32" t="s">
+      <c r="B13" s="47"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30" t="s">
         <v>148</v>
       </c>
-      <c r="F13" s="32" t="s">
+      <c r="F13" s="30" t="s">
         <v>149</v>
       </c>
-      <c r="G13" s="41" t="s">
+      <c r="G13" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="H13" s="32" t="s">
+      <c r="H13" s="30" t="s">
         <v>150</v>
       </c>
-      <c r="I13" s="42">
+      <c r="I13" s="40">
         <v>271</v>
       </c>
     </row>
     <row r="14" ht="57">
-      <c r="A14" s="36" t="s">
+      <c r="A14" s="34" t="s">
         <v>151</v>
       </c>
-      <c r="B14" s="37" t="s">
+      <c r="B14" s="35" t="s">
         <v>109</v>
       </c>
-      <c r="C14" s="38">
+      <c r="C14" s="36">
         <v>45380</v>
       </c>
-      <c r="D14" s="39" t="s">
+      <c r="D14" s="37" t="s">
         <v>152</v>
       </c>
-      <c r="E14" s="40" t="s">
+      <c r="E14" s="38" t="s">
         <v>153</v>
       </c>
-      <c r="F14" s="40" t="s">
+      <c r="F14" s="38" t="s">
         <v>154</v>
       </c>
-      <c r="G14" s="41" t="s">
+      <c r="G14" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="40" t="s">
+      <c r="H14" s="38" t="s">
         <v>155</v>
       </c>
-      <c r="I14" s="42">
+      <c r="I14" s="40">
         <v>272</v>
       </c>
     </row>
     <row r="15" ht="99.75">
-      <c r="A15" s="36" t="s">
+      <c r="A15" s="34" t="s">
         <v>156</v>
       </c>
-      <c r="B15" s="43"/>
-      <c r="C15" s="44"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="40" t="s">
+      <c r="B15" s="41"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="43"/>
+      <c r="E15" s="38" t="s">
         <v>157</v>
       </c>
-      <c r="F15" s="40" t="s">
+      <c r="F15" s="38" t="s">
         <v>158</v>
       </c>
-      <c r="G15" s="41" t="s">
+      <c r="G15" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="H15" s="40" t="s">
+      <c r="H15" s="38" t="s">
         <v>159</v>
       </c>
-      <c r="I15" s="42">
+      <c r="I15" s="40">
         <v>273</v>
       </c>
     </row>
     <row r="16" ht="85.5">
-      <c r="A16" s="36" t="s">
+      <c r="A16" s="34" t="s">
         <v>151</v>
       </c>
-      <c r="B16" s="37" t="s">
+      <c r="B16" s="35" t="s">
         <v>109</v>
       </c>
-      <c r="C16" s="38">
+      <c r="C16" s="36">
         <v>43235</v>
       </c>
-      <c r="D16" s="39" t="s">
+      <c r="D16" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="E16" s="40" t="s">
+      <c r="E16" s="38" t="s">
         <v>161</v>
       </c>
-      <c r="F16" s="40" t="s">
+      <c r="F16" s="38" t="s">
         <v>162</v>
       </c>
-      <c r="G16" s="41" t="s">
+      <c r="G16" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="H16" s="40" t="s">
+      <c r="H16" s="38" t="s">
         <v>163</v>
       </c>
-      <c r="I16" s="42">
+      <c r="I16" s="40">
         <v>274</v>
       </c>
     </row>
@@ -3061,264 +3165,258 @@
       <c r="A17" s="36" t="s">
         <v>156</v>
       </c>
-      <c r="B17" s="43"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="45"/>
-      <c r="E17" s="40" t="s">
+      <c r="B17" s="48"/>
+      <c r="C17" s="49"/>
+      <c r="D17" s="50"/>
+      <c r="E17" s="37" t="s">
         <v>164</v>
       </c>
-      <c r="F17" s="40" t="s">
+      <c r="F17" s="37" t="s">
         <v>165</v>
       </c>
-      <c r="G17" s="41" t="s">
+      <c r="G17" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="H17" s="40" t="s">
+      <c r="H17" s="37" t="s">
         <v>166</v>
       </c>
-      <c r="I17" s="42">
+      <c r="I17" s="40">
         <v>275</v>
       </c>
     </row>
-    <row r="18" ht="14.25">
-      <c r="A18" s="31"/>
-      <c r="B18" s="31"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="31"/>
-      <c r="H18" s="32"/>
-      <c r="I18" s="31"/>
-    </row>
-    <row r="19" ht="14.25">
-      <c r="A19" s="31"/>
-      <c r="B19" s="31"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="32"/>
-      <c r="E19" s="32"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="31"/>
-      <c r="H19" s="32"/>
-      <c r="I19" s="31"/>
-    </row>
-    <row r="20" ht="14.25">
-      <c r="A20" s="31"/>
-      <c r="B20" s="31"/>
-      <c r="C20" s="31"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="32"/>
-      <c r="F20" s="32"/>
-      <c r="G20" s="31"/>
-      <c r="H20" s="32"/>
+    <row r="18" ht="114">
+      <c r="A18" s="52" t="s">
+        <v>167</v>
+      </c>
+      <c r="B18" s="53" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" s="54" t="s">
+        <v>168</v>
+      </c>
+      <c r="D18" s="55" t="s">
+        <v>169</v>
+      </c>
+      <c r="E18" s="55" t="s">
+        <v>170</v>
+      </c>
+      <c r="F18" s="55" t="s">
+        <v>171</v>
+      </c>
+      <c r="G18" s="56" t="s">
+        <v>172</v>
+      </c>
+      <c r="H18" s="55" t="s">
+        <v>173</v>
+      </c>
+      <c r="I18" s="40">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="19" ht="99.75">
+      <c r="A19" s="52" t="s">
+        <v>174</v>
+      </c>
+      <c r="B19" s="53"/>
+      <c r="C19" s="54"/>
+      <c r="D19" s="55" t="s">
+        <v>169</v>
+      </c>
+      <c r="E19" s="55" t="s">
+        <v>175</v>
+      </c>
+      <c r="F19" s="55" t="s">
+        <v>176</v>
+      </c>
+      <c r="G19" s="56" t="s">
+        <v>177</v>
+      </c>
+      <c r="H19" s="55" t="s">
+        <v>178</v>
+      </c>
+      <c r="I19" s="40">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="20" ht="114">
+      <c r="A20" s="52" t="s">
+        <v>179</v>
+      </c>
+      <c r="B20" s="53"/>
+      <c r="C20" s="54"/>
+      <c r="D20" s="55" t="s">
+        <v>169</v>
+      </c>
+      <c r="E20" s="55" t="s">
+        <v>180</v>
+      </c>
+      <c r="F20" s="55" t="s">
+        <v>181</v>
+      </c>
+      <c r="G20" s="56" t="s">
+        <v>182</v>
+      </c>
+      <c r="H20" s="55" t="s">
+        <v>183</v>
+      </c>
+      <c r="I20" s="29">
+        <v>278</v>
+      </c>
     </row>
     <row r="21" ht="14.25">
-      <c r="A21" s="31"/>
-      <c r="B21" s="31"/>
-      <c r="C21" s="31"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="31"/>
-      <c r="H21" s="32"/>
+      <c r="A21" s="29"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="30"/>
+      <c r="F21" s="30"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="30"/>
     </row>
     <row r="22" ht="14.25">
-      <c r="A22" s="31"/>
-      <c r="B22" s="31"/>
-      <c r="C22" s="31"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="32"/>
-      <c r="F22" s="32"/>
-      <c r="G22" s="31"/>
-      <c r="H22" s="32"/>
+      <c r="A22" s="29"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="30"/>
     </row>
     <row r="23" ht="21.75">
-      <c r="A23" s="50"/>
-      <c r="B23" s="50"/>
-      <c r="C23" s="50"/>
-      <c r="D23" s="50"/>
-      <c r="E23" s="50"/>
-      <c r="F23" s="50"/>
-      <c r="G23" s="50"/>
-      <c r="H23" s="50"/>
-    </row>
-    <row r="24" ht="21.75">
-      <c r="A24" s="51"/>
-      <c r="B24" s="51"/>
-      <c r="C24" s="51"/>
-      <c r="D24" s="51"/>
-      <c r="E24" s="51"/>
-      <c r="F24" s="51"/>
-      <c r="G24" s="51"/>
-      <c r="H24" s="51"/>
-    </row>
-    <row r="25" ht="21.75">
-      <c r="A25" s="51"/>
-      <c r="B25" s="32"/>
-      <c r="C25" s="32"/>
-      <c r="D25" s="32"/>
-      <c r="E25" s="51"/>
-      <c r="F25" s="51"/>
-      <c r="G25" s="51"/>
-      <c r="H25" s="51"/>
-    </row>
-    <row r="26" ht="21.75">
-      <c r="A26" s="51"/>
-      <c r="B26" s="51"/>
-      <c r="C26" s="51"/>
-      <c r="D26" s="51"/>
-      <c r="E26" s="51"/>
-      <c r="F26" s="51"/>
-      <c r="G26" s="51"/>
-      <c r="H26" s="51"/>
-    </row>
-    <row r="27" ht="21.75">
-      <c r="A27" s="51"/>
-      <c r="B27" s="32"/>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="51"/>
-      <c r="F27" s="51"/>
-      <c r="G27" s="51"/>
-      <c r="H27" s="51"/>
+      <c r="A23" s="57"/>
+      <c r="B23" s="58"/>
+      <c r="C23" s="58"/>
+      <c r="D23" s="58"/>
+      <c r="E23" s="58"/>
+      <c r="F23" s="58"/>
+      <c r="G23" s="58"/>
+      <c r="H23" s="57"/>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="A24" s="29"/>
+      <c r="B24" s="29"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="29"/>
+      <c r="H24" s="30"/>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="A25" s="29"/>
+      <c r="B25" s="29"/>
+      <c r="C25" s="29"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="30"/>
+      <c r="F25" s="30"/>
+      <c r="G25" s="29"/>
+      <c r="H25" s="30"/>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="A26" s="29"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="30"/>
+      <c r="E26" s="30"/>
+      <c r="F26" s="30"/>
+      <c r="G26" s="29"/>
+      <c r="H26" s="30"/>
+    </row>
+    <row r="27" ht="14.25">
+      <c r="A27" s="29"/>
+      <c r="B27" s="29"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="30"/>
+      <c r="E27" s="30"/>
+      <c r="F27" s="30"/>
+      <c r="G27" s="29"/>
+      <c r="H27" s="30"/>
     </row>
     <row r="28" ht="14.25">
-      <c r="A28" s="42"/>
-      <c r="B28" s="31"/>
-      <c r="C28" s="31"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="31"/>
-      <c r="H28" s="32"/>
+      <c r="A28" s="29"/>
+      <c r="B28" s="29"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="29"/>
+      <c r="H28" s="30"/>
     </row>
     <row r="29" ht="14.25">
-      <c r="A29" s="31"/>
-      <c r="B29" s="31"/>
-      <c r="C29" s="31"/>
-      <c r="D29" s="32"/>
-      <c r="E29" s="32"/>
-      <c r="F29" s="32"/>
-      <c r="G29" s="31"/>
-      <c r="H29" s="32"/>
+      <c r="A29" s="29"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="30"/>
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="29"/>
+      <c r="H29" s="30"/>
     </row>
     <row r="30" ht="14.25">
-      <c r="A30" s="31"/>
-      <c r="B30" s="31"/>
-      <c r="C30" s="31"/>
-      <c r="D30" s="32"/>
-      <c r="E30" s="32"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="31"/>
-      <c r="H30" s="32"/>
+      <c r="A30" s="29"/>
+      <c r="B30" s="29"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="30"/>
+      <c r="E30" s="30"/>
+      <c r="F30" s="30"/>
+      <c r="G30" s="29"/>
+      <c r="H30" s="30"/>
     </row>
     <row r="31" ht="14.25">
-      <c r="A31" s="31"/>
-      <c r="B31" s="31"/>
-      <c r="C31" s="31"/>
-      <c r="D31" s="32"/>
-      <c r="E31" s="32"/>
-      <c r="F31" s="32"/>
-      <c r="G31" s="31"/>
-      <c r="H31" s="32"/>
+      <c r="A31" s="29"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="30"/>
+      <c r="E31" s="30"/>
+      <c r="F31" s="30"/>
+      <c r="G31" s="29"/>
+      <c r="H31" s="30"/>
     </row>
     <row r="32" ht="14.25">
-      <c r="A32" s="31"/>
-      <c r="B32" s="31"/>
-      <c r="C32" s="31"/>
-      <c r="D32" s="32"/>
-      <c r="E32" s="32"/>
-      <c r="F32" s="32"/>
-      <c r="G32" s="31"/>
-      <c r="H32" s="32"/>
+      <c r="A32" s="29"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="30"/>
+      <c r="E32" s="30"/>
+      <c r="F32" s="30"/>
+      <c r="G32" s="29"/>
+      <c r="H32" s="30"/>
     </row>
     <row r="33" ht="14.25">
-      <c r="A33" s="31"/>
-      <c r="B33" s="31"/>
-      <c r="C33" s="31"/>
-      <c r="D33" s="32"/>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="31"/>
-      <c r="H33" s="32"/>
+      <c r="A33" s="29"/>
+      <c r="B33" s="29"/>
+      <c r="C33" s="29"/>
+      <c r="D33" s="30"/>
+      <c r="E33" s="30"/>
+      <c r="F33" s="30"/>
+      <c r="G33" s="29"/>
+      <c r="H33" s="30"/>
     </row>
     <row r="34" ht="14.25">
-      <c r="A34" s="31"/>
-      <c r="B34" s="31"/>
-      <c r="C34" s="31"/>
-      <c r="D34" s="32"/>
-      <c r="E34" s="32"/>
-      <c r="F34" s="32"/>
-      <c r="G34" s="31"/>
-      <c r="H34" s="32"/>
+      <c r="A34" s="29"/>
+      <c r="B34" s="29"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="30"/>
+      <c r="E34" s="30"/>
+      <c r="F34" s="30"/>
+      <c r="G34" s="29"/>
+      <c r="H34" s="30"/>
     </row>
     <row r="35" ht="14.25">
-      <c r="A35" s="31"/>
+      <c r="A35" s="29"/>
     </row>
     <row r="36" ht="14.25">
-      <c r="A36" s="31"/>
+      <c r="A36" s="29"/>
     </row>
     <row r="37" ht="14.25">
-      <c r="A37" s="31"/>
+      <c r="A37" s="29"/>
     </row>
     <row r="38" ht="14.25">
-      <c r="A38" s="31"/>
-    </row>
-    <row r="39" ht="14.25">
-      <c r="A39" s="31"/>
-    </row>
-    <row r="40" ht="14.25">
-      <c r="A40" s="31"/>
-    </row>
-    <row r="41" ht="14.25">
-      <c r="A41" s="31"/>
-      <c r="B41" s="31"/>
-      <c r="C41" s="31"/>
-      <c r="D41" s="32"/>
-      <c r="E41" s="32"/>
-      <c r="F41" s="32"/>
-      <c r="G41" s="31"/>
-      <c r="H41" s="32"/>
-    </row>
-    <row r="42" ht="14.25">
-      <c r="A42" s="31"/>
-      <c r="B42" s="31"/>
-      <c r="C42" s="31"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="32"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="31"/>
-      <c r="H42" s="32"/>
-    </row>
-    <row r="43" ht="14.25">
-      <c r="A43" s="31"/>
-      <c r="E43" s="32"/>
-      <c r="F43" s="32"/>
-      <c r="G43" s="31"/>
-      <c r="H43" s="32"/>
-    </row>
-    <row r="44" ht="14.25">
-      <c r="A44" s="31"/>
-      <c r="B44" s="31"/>
-      <c r="C44" s="31"/>
-      <c r="D44" s="32"/>
-      <c r="E44" s="32"/>
-      <c r="F44" s="32"/>
-      <c r="G44" s="31"/>
-      <c r="H44" s="32"/>
-    </row>
-    <row r="45" ht="14.25">
-      <c r="A45" s="31"/>
-      <c r="E45" s="32"/>
-      <c r="F45" s="32"/>
-      <c r="G45" s="31"/>
-      <c r="H45" s="32"/>
-    </row>
-    <row r="46" ht="14.25">
-      <c r="A46" s="31"/>
+      <c r="A38" s="29"/>
     </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="26">
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
@@ -3343,6 +3441,8 @@
     <mergeCell ref="B16:B17"/>
     <mergeCell ref="C16:C17"/>
     <mergeCell ref="D16:D17"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="C18:C20"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>